<commit_message>
Schrap de vijf vragen met antwoord nul
Ze ontbraken in de eerdere schrapronde omdat ze wel een bruikbare bron hadden.
Nul maakt elke deling stuk en verandert bij optellen niets, dus in een rekenspel
zijn ze onbruikbaar hoe juist het antwoord ook is.

Vier zijn ook inhoudelijk kapot; een bevat letterlijk de correctie van de
schrijver. De vijfde is juist perfect gesteld — het vriespunt van water is nul
graden — en sneuvelt puur op de rekenkunde.

Bank en reviewblad staan nu op 1411.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vragen/geschrapte_vragen.xlsx
+++ b/vragen/geschrapte_vragen.xlsx
@@ -9,9 +9,7 @@
   <sheets>
     <sheet name="Geschrapt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Geschrapt'!$A$1:$S$41</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,28 +28,13 @@
     <font>
       <b val="1"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <sz val="10"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F3864"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -72,19 +55,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -451,2337 +425,2636 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S41"/>
+  <dimension ref="A1:S46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="74" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-  </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Nr</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>In gebruik</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Categorie</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Categorie (was)</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Vraag NL</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Vraag EN (zoekhulp)</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Antwoord</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Bron (bestaand)</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Bron (jouw aanvulling)</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Commons-fotolink</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Verwijderen</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Advies Claude</t>
         </is>
       </c>
-      <c r="M1" s="2" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Jouw opmerking</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Let op</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Bron (geverifieerd)</t>
         </is>
       </c>
-      <c r="P1" s="2" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Bewijszin</t>
         </is>
       </c>
-      <c r="Q1" s="2" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Controle</t>
         </is>
       </c>
-      <c r="R1" s="2" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Vertrouwen bron</t>
         </is>
       </c>
-      <c r="S1" s="2" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Status oude bron</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" t="n">
         <v>68</v>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>daily</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Hoe lang waren de langste mouwen aan een kledingstuk ooit in meters?</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>How long were the longest sleeves on a garment ever in metres?</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G2" t="n">
         <v>51</v>
       </c>
-      <c r="H2" s="3" t="inlineStr"/>
-      <c r="I2" s="3" t="inlineStr"/>
-      <c r="J2" s="3" t="inlineStr"/>
-      <c r="K2" s="3" t="inlineStr"/>
-      <c r="L2" s="3" t="inlineStr"/>
-      <c r="M2" s="3" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr">
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O2" s="3" t="inlineStr"/>
-      <c r="P2" s="4" t="inlineStr"/>
-      <c r="Q2" s="3" t="inlineStr"/>
-      <c r="R2" s="3" t="inlineStr"/>
-      <c r="S2" s="3" t="inlineStr">
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" t="n">
         <v>188</v>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Hoeveel minuten kook je een ei voor een zacht gekookt ei?</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>How many minutes do you cook an egg for a soft boiled egg?</t>
         </is>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="G3" t="n">
         <v>6</v>
       </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr"/>
-      <c r="J3" s="3" t="inlineStr"/>
-      <c r="K3" s="3" t="inlineStr"/>
-      <c r="L3" s="3" t="inlineStr"/>
-      <c r="M3" s="3" t="inlineStr"/>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr"/>
-      <c r="Q3" s="3" t="inlineStr"/>
-      <c r="R3" s="3" t="inlineStr"/>
-      <c r="S3" s="3" t="inlineStr">
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+      <c r="S3" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" t="n">
         <v>189</v>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Hoeveel rundvleesburgers verkocht McDonald’s wereldwijd in 2023?</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>How many beef burgers sold McDonalds worldwide in 2023?</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="G4" t="n">
         <v>44000000000</v>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>https://corporate.mcdonalds.com/corpmcd/our-company/annual-reports.html</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr"/>
-      <c r="J4" s="3" t="inlineStr"/>
-      <c r="K4" s="3" t="inlineStr"/>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr"/>
-      <c r="N4" s="4" t="inlineStr"/>
-      <c r="O4" s="3" t="inlineStr"/>
-      <c r="P4" s="4" t="inlineStr">
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
         <is>
           <t>McDonald's telt sinds 1994 geen verkochte hamburgers meer en publiceert dit getal niet. Schattingen liggen tussen 2,4 en 6,5 miljard per jaar; 44 miljard is een orde van grootte te hoog.</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr"/>
-      <c r="R4" s="3" t="inlineStr"/>
-      <c r="S4" s="3" t="inlineStr">
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+      <c r="S4" t="inlineStr">
         <is>
           <t>geen bron mogelijk (fout)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" t="n">
         <v>284</v>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Geografie</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Geografie</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Hoeveel landen liggen volledig op het zuidelijk halfrond?</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>How many countries are in the southern hemisphere?</t>
         </is>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="G5" t="n">
         <v>32</v>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>World Atlas is not definitive; classification depends on boundary convention.</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr"/>
-      <c r="J5" s="3" t="inlineStr"/>
-      <c r="K5" s="3" t="inlineStr"/>
-      <c r="L5" s="3" t="inlineStr"/>
-      <c r="M5" s="3" t="inlineStr"/>
-      <c r="N5" s="4" t="inlineStr"/>
-      <c r="O5" s="3" t="inlineStr"/>
-      <c r="P5" s="4" t="inlineStr">
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
         <is>
           <t>Het antwoord hangt af van de gekozen grensconventie; de oorspronkelijke bron zei dat zelf al. Geen vaste telling mogelijk.</t>
         </is>
       </c>
-      <c r="Q5" s="3" t="inlineStr"/>
-      <c r="R5" s="3" t="inlineStr"/>
-      <c r="S5" s="3" t="inlineStr">
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+      <c r="S5" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" t="n">
         <v>381</v>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Mode en lifestyle</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>Mode en lifestyle</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Hoeveel centimeter lang is een standaard das bij het strikken?</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>How many centimeters is a standard tie when you tie?</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="G6" t="n">
         <v>145</v>
       </c>
-      <c r="H6" s="3" t="inlineStr"/>
-      <c r="I6" s="3" t="inlineStr"/>
-      <c r="J6" s="3" t="inlineStr"/>
-      <c r="K6" s="3" t="inlineStr"/>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr"/>
-      <c r="N6" s="4" t="inlineStr">
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O6" s="3" t="inlineStr"/>
-      <c r="P6" s="4" t="inlineStr"/>
-      <c r="Q6" s="3" t="inlineStr"/>
-      <c r="R6" s="3" t="inlineStr"/>
-      <c r="S6" s="3" t="inlineStr">
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" t="n">
         <v>382</v>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Mode en lifestyle</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Mode en lifestyle</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Hoeveel gaten heeft een standaard schoenveter meestal in één schoen?</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>How many holes does a standard shoelace usually have in one shoe?</t>
         </is>
       </c>
-      <c r="G7" s="3" t="n">
+      <c r="G7" t="n">
         <v>12</v>
       </c>
-      <c r="H7" s="3" t="inlineStr"/>
-      <c r="I7" s="3" t="inlineStr"/>
-      <c r="J7" s="3" t="inlineStr"/>
-      <c r="K7" s="3" t="inlineStr"/>
-      <c r="L7" s="3" t="inlineStr"/>
-      <c r="M7" s="3" t="inlineStr"/>
-      <c r="N7" s="4" t="inlineStr">
+      <c r="H7" t="inlineStr"/>
+      <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O7" s="3" t="inlineStr"/>
-      <c r="P7" s="4" t="inlineStr"/>
-      <c r="Q7" s="3" t="inlineStr"/>
-      <c r="R7" s="3" t="inlineStr"/>
-      <c r="S7" s="3" t="inlineStr">
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" t="n">
         <v>384</v>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Mode en lifestyle</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>Mode en lifestyle</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Hoeveel millimeter breed is een standaard herenhorlogeband?</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>How many millimeters wide is a standard men's watch band?</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="G8" t="n">
         <v>22</v>
       </c>
-      <c r="H8" s="3" t="inlineStr"/>
-      <c r="I8" s="3" t="inlineStr"/>
-      <c r="J8" s="3" t="inlineStr"/>
-      <c r="K8" s="3" t="inlineStr"/>
-      <c r="L8" s="3" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
-      <c r="N8" s="4" t="inlineStr">
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O8" s="3" t="inlineStr"/>
-      <c r="P8" s="4" t="inlineStr"/>
-      <c r="Q8" s="3" t="inlineStr"/>
-      <c r="R8" s="3" t="inlineStr"/>
-      <c r="S8" s="3" t="inlineStr">
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" t="n">
         <v>446</v>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Hoe lang was de langste snoepstaaf ooit in kilometer?</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>How long was the longest candy bar ever in kilometres?</t>
         </is>
       </c>
-      <c r="G9" s="3" t="n">
+      <c r="G9" t="n">
         <v>1</v>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
-      <c r="I9" s="3" t="inlineStr"/>
-      <c r="J9" s="3" t="inlineStr"/>
-      <c r="K9" s="3" t="inlineStr"/>
-      <c r="L9" s="3" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
-      <c r="N9" s="4" t="inlineStr">
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O9" s="3" t="inlineStr"/>
-      <c r="P9" s="4" t="inlineStr"/>
-      <c r="Q9" s="3" t="inlineStr"/>
-      <c r="R9" s="3" t="inlineStr"/>
-      <c r="S9" s="3" t="inlineStr">
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" t="n">
         <v>451</v>
       </c>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Hoeveel kilometer was de langste zwemtocht ooit?</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>How many kilometres was the longest swim ever?</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="G10" t="n">
         <v>500</v>
       </c>
-      <c r="H10" s="3" t="inlineStr"/>
-      <c r="I10" s="3" t="inlineStr"/>
-      <c r="J10" s="3" t="inlineStr"/>
-      <c r="K10" s="3" t="inlineStr"/>
-      <c r="L10" s="3" t="inlineStr"/>
-      <c r="M10" s="3" t="inlineStr"/>
-      <c r="N10" s="4" t="inlineStr">
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O10" s="3" t="inlineStr"/>
-      <c r="P10" s="4" t="inlineStr"/>
-      <c r="Q10" s="3" t="inlineStr"/>
-      <c r="R10" s="3" t="inlineStr"/>
-      <c r="S10" s="3" t="inlineStr">
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" t="n">
         <v>457</v>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>puzzel</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>Records en vergelijkingen</t>
         </is>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Hoeveel voertuigen stonden er ongeveer in de langste file ooit?</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>How many vehicles were in the longest traffic traffic ever?</t>
         </is>
       </c>
-      <c r="G11" s="3" t="n">
+      <c r="G11" t="n">
         <v>12000</v>
       </c>
-      <c r="H11" s="3" t="inlineStr"/>
-      <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="3" t="inlineStr"/>
-      <c r="K11" s="3" t="inlineStr"/>
-      <c r="L11" s="3" t="inlineStr"/>
-      <c r="M11" s="3" t="inlineStr"/>
-      <c r="N11" s="4" t="inlineStr">
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O11" s="3" t="inlineStr"/>
-      <c r="P11" s="4" t="inlineStr"/>
-      <c r="Q11" s="3" t="inlineStr"/>
-      <c r="R11" s="3" t="inlineStr"/>
-      <c r="S11" s="3" t="inlineStr">
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" t="n">
         <v>633</v>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
         <is>
           <t>Landbouw en industrie</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" t="inlineStr">
         <is>
           <t>Dieren</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Hoeveel bijenkorven produceert de gemiddelde Ethiopische bijenhouder per jaar?</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr"/>
-      <c r="G12" s="3" t="n">
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="3" t="inlineStr"/>
-      <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="3" t="inlineStr"/>
-      <c r="K12" s="3" t="inlineStr"/>
-      <c r="L12" s="3" t="inlineStr"/>
-      <c r="M12" s="3" t="inlineStr"/>
-      <c r="N12" s="4" t="inlineStr">
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O12" s="3" t="inlineStr"/>
-      <c r="P12" s="4" t="inlineStr"/>
-      <c r="Q12" s="3" t="inlineStr"/>
-      <c r="R12" s="3" t="inlineStr"/>
-      <c r="S12" s="3" t="inlineStr">
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" t="n">
         <v>638</v>
       </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
         <is>
           <t>Dieren</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D13" t="inlineStr">
         <is>
           <t>Dieren</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Hoeveel eieren legt een kangoeroe per worp?</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr"/>
-      <c r="G13" s="3" t="n">
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="3" t="inlineStr"/>
-      <c r="I13" s="3" t="inlineStr"/>
-      <c r="J13" s="3" t="inlineStr"/>
-      <c r="K13" s="3" t="inlineStr"/>
-      <c r="L13" s="3" t="inlineStr"/>
-      <c r="M13" s="3" t="inlineStr"/>
-      <c r="N13" s="4" t="inlineStr">
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O13" s="3" t="inlineStr"/>
-      <c r="P13" s="4" t="inlineStr"/>
-      <c r="Q13" s="3" t="inlineStr"/>
-      <c r="R13" s="3" t="inlineStr"/>
-      <c r="S13" s="3" t="inlineStr">
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" t="n">
         <v>688</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>Dieren</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Dieren</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Hoeveel van de 10 giftigste slangen ter wereld komen voor in Australië?</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr"/>
-      <c r="G14" s="3" t="n">
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="n">
         <v>0</v>
       </c>
-      <c r="H14" s="3" t="inlineStr"/>
-      <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="3" t="inlineStr"/>
-      <c r="K14" s="3" t="inlineStr"/>
-      <c r="L14" s="3" t="inlineStr"/>
-      <c r="M14" s="3" t="inlineStr"/>
-      <c r="N14" s="4" t="inlineStr">
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O14" s="3" t="inlineStr"/>
-      <c r="P14" s="4" t="inlineStr"/>
-      <c r="Q14" s="3" t="inlineStr"/>
-      <c r="R14" s="3" t="inlineStr"/>
-      <c r="S14" s="3" t="inlineStr">
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" t="n">
         <v>708</v>
       </c>
-      <c r="B15" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D15" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Hoeveel gram weegt een standaard chocoladereep vaak?</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>How many grams does a standard chocolate bar often weigh?</t>
         </is>
       </c>
-      <c r="G15" s="3" t="n">
+      <c r="G15" t="n">
         <v>100</v>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>No universal standard; depends on product and market.</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="3" t="inlineStr"/>
-      <c r="K15" s="3" t="inlineStr"/>
-      <c r="L15" s="3" t="inlineStr"/>
-      <c r="M15" s="3" t="inlineStr"/>
-      <c r="N15" s="4" t="inlineStr"/>
-      <c r="O15" s="3" t="inlineStr"/>
-      <c r="P15" s="4" t="inlineStr">
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
         <is>
           <t>Chocoladerepen hebben geen standaardgewicht; het verschilt per merk en land.</t>
         </is>
       </c>
-      <c r="Q15" s="3" t="inlineStr"/>
-      <c r="R15" s="3" t="inlineStr"/>
-      <c r="S15" s="3" t="inlineStr">
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" t="n">
         <v>769</v>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>Filosofie, psychologie en religie</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" t="inlineStr">
         <is>
           <t>Filosofie, psychologie en religie</t>
         </is>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Hoeveel zwaarden waren er volgens de legende van koning Arthur beschikbaar?</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>How many swords were available according to King Arthur's legend?</t>
         </is>
       </c>
-      <c r="G16" s="3" t="n">
+      <c r="G16" t="n">
         <v>1</v>
       </c>
-      <c r="H16" s="3" t="inlineStr"/>
-      <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="3" t="inlineStr"/>
-      <c r="K16" s="3" t="inlineStr"/>
-      <c r="L16" s="3" t="inlineStr"/>
-      <c r="M16" s="3" t="inlineStr"/>
-      <c r="N16" s="4" t="inlineStr">
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O16" s="3" t="inlineStr"/>
-      <c r="P16" s="4" t="inlineStr"/>
-      <c r="Q16" s="3" t="inlineStr"/>
-      <c r="R16" s="3" t="inlineStr"/>
-      <c r="S16" s="3" t="inlineStr">
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" t="n">
         <v>806</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
         <is>
           <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="D17" t="inlineStr">
         <is>
           <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Hoeveel piramides staan er ongeveer in Gizeh?</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>How many pyramids are there in Giza?</t>
         </is>
       </c>
-      <c r="G17" s="3" t="n">
+      <c r="G17" t="n">
         <v>3</v>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="H17" t="inlineStr">
         <is>
           <t>https://www.britannica.com/place/Pyramids-of-Giza</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="3" t="inlineStr"/>
-      <c r="K17" s="3" t="inlineStr"/>
-      <c r="L17" s="3" t="inlineStr"/>
-      <c r="M17" s="3" t="inlineStr"/>
-      <c r="N17" s="4" t="inlineStr"/>
-      <c r="O17" s="3" t="inlineStr">
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
         <is>
           <t>https://en.wikipedia.org/wiki/Giza_pyramid_complex</t>
         </is>
       </c>
-      <c r="P17" s="4" t="inlineStr">
+      <c r="P17" t="inlineStr">
         <is>
           <t>Dubbel met vraag 241, en "ongeveer" past niet bij een exact getal. Gizeh telt drie hoofdpiramides maar met de koninginnenpiramides erbij negen.</t>
         </is>
       </c>
-      <c r="Q17" s="3" t="inlineStr"/>
-      <c r="R17" s="3" t="inlineStr">
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr">
         <is>
           <t>onbruikbaar</t>
         </is>
       </c>
-      <c r="S17" s="3" t="inlineStr">
+      <c r="S17" t="inlineStr">
         <is>
           <t>vraag deugt niet, zie toelichting</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" t="n">
         <v>808</v>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
         <is>
           <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" t="inlineStr">
         <is>
           <t>Gebouwen en infrastructuur</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Hoeveel rivieren bruggen telt Sydney Harbour?</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr"/>
-      <c r="G18" s="3" t="n">
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="n">
         <v>0</v>
       </c>
-      <c r="H18" s="3" t="inlineStr"/>
-      <c r="I18" s="3" t="inlineStr"/>
-      <c r="J18" s="3" t="inlineStr"/>
-      <c r="K18" s="3" t="inlineStr"/>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
         <is>
           <t>Onleesbaar: "rivieren bruggen telt Sydney Harbour".</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr"/>
-      <c r="N18" s="4" t="inlineStr">
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O18" s="3" t="inlineStr"/>
-      <c r="P18" s="4" t="inlineStr"/>
-      <c r="Q18" s="3" t="inlineStr"/>
-      <c r="R18" s="3" t="inlineStr"/>
-      <c r="S18" s="3" t="inlineStr">
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+      <c r="S18" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" t="n">
         <v>837</v>
       </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>Geografie</t>
         </is>
       </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Geografie</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>Hoeveel Europese landen liggen er niet op het vasteland (exclusief eilanden) in de EU als eilandstaten?</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>How many European countries are not on the mainland (excluding islands) in the EU as island states?</t>
         </is>
       </c>
-      <c r="G19" s="3" t="n">
+      <c r="G19" t="n">
         <v>2</v>
       </c>
-      <c r="H19" s="3" t="inlineStr"/>
-      <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="3" t="inlineStr"/>
-      <c r="K19" s="3" t="inlineStr"/>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
         <is>
           <t>Onleesbaar geformuleerd ("liggen er niet op het vasteland (exclusief eilanden) als eilandstaten").</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr"/>
-      <c r="N19" s="4" t="inlineStr">
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O19" s="3" t="inlineStr"/>
-      <c r="P19" s="4" t="inlineStr">
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
         <is>
           <t>De vraag spreekt zichzelf tegen: "niet op het vasteland (exclusief eilanden)". Bovendien zijn Ierland, Malta en Cyprus alle drie eilandstaten in de EU, dus het antwoord twee klopt hoe dan ook niet.</t>
         </is>
       </c>
-      <c r="Q19" s="3" t="inlineStr"/>
-      <c r="R19" s="3" t="inlineStr"/>
-      <c r="S19" s="3" t="inlineStr">
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+      <c r="S19" t="inlineStr">
         <is>
           <t>vraag deugt niet (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" t="n">
         <v>1116</v>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
         <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Hoeveel snaarinstrumenten bevat de klassieke Japanse koto-ensemble van hoort?</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>How many string instruments does the classic Japanese koto ensemble contain?</t>
         </is>
       </c>
-      <c r="G20" s="3" t="n">
+      <c r="G20" t="n">
         <v>13</v>
       </c>
-      <c r="H20" s="3" t="inlineStr"/>
-      <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="3" t="inlineStr"/>
-      <c r="K20" s="3" t="inlineStr"/>
-      <c r="L20" s="3" t="inlineStr">
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
         <is>
           <t>Onafgemaakte zin: "koto-ensemble van hoort".</t>
         </is>
       </c>
-      <c r="M20" s="3" t="inlineStr"/>
-      <c r="N20" s="4" t="inlineStr">
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O20" s="3" t="inlineStr"/>
-      <c r="P20" s="4" t="inlineStr"/>
-      <c r="Q20" s="3" t="inlineStr"/>
-      <c r="R20" s="3" t="inlineStr"/>
-      <c r="S20" s="3" t="inlineStr">
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr"/>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+      <c r="S20" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" t="n">
         <v>1119</v>
       </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
         <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" t="inlineStr">
         <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>Hoeveel snaren heeft de West-Afrikaanse djembé als trommel?</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr"/>
-      <c r="G21" s="3" t="n">
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
         <v>0</v>
       </c>
-      <c r="H21" s="3" t="inlineStr"/>
-      <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="3" t="inlineStr"/>
-      <c r="K21" s="3" t="inlineStr"/>
-      <c r="L21" s="3" t="inlineStr">
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
         <is>
           <t>Feitelijk onjuist: een djembé is een trommel en heeft geen snaren.</t>
         </is>
       </c>
-      <c r="M21" s="3" t="inlineStr"/>
-      <c r="N21" s="4" t="inlineStr">
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O21" s="3" t="inlineStr"/>
-      <c r="P21" s="4" t="inlineStr"/>
-      <c r="Q21" s="3" t="inlineStr"/>
-      <c r="R21" s="3" t="inlineStr"/>
-      <c r="S21" s="3" t="inlineStr">
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr"/>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+      <c r="S21" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="n">
+      <c r="A22" t="n">
         <v>1124</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
         <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Hoeveel snaren heeft de klassieke Mexicaanse mariachi-gitarron (bajo sexto)?</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>How many strings does the classic Mexican mariachi-gitarron (bajo sexto) have?</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n">
+      <c r="G22" t="n">
         <v>12</v>
       </c>
-      <c r="H22" s="3" t="inlineStr"/>
-      <c r="I22" s="3" t="inlineStr"/>
-      <c r="J22" s="3" t="inlineStr"/>
-      <c r="K22" s="3" t="inlineStr"/>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
         <is>
           <t>Verwart twee instrumenten: een guitarrón is geen bajo sexto.</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr"/>
-      <c r="N22" s="4" t="inlineStr">
+      <c r="M22" t="inlineStr"/>
+      <c r="N22" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O22" s="3" t="inlineStr"/>
-      <c r="P22" s="4" t="inlineStr"/>
-      <c r="Q22" s="3" t="inlineStr"/>
-      <c r="R22" s="3" t="inlineStr"/>
-      <c r="S22" s="3" t="inlineStr">
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr"/>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+      <c r="S22" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="n">
+      <c r="A23" t="n">
         <v>1146</v>
       </c>
-      <c r="B23" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>Dagelijks leven</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E23" s="4" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Hoeveel NL-postcodes cijfers heeft een Nederlandse postcode standaard (vier cijfers plus twee letters)?</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>How many NL postal code numbers has a Dutch postal code standard (four digits plus two letters)?</t>
         </is>
       </c>
-      <c r="G23" s="3" t="n">
+      <c r="G23" t="n">
         <v>4</v>
       </c>
-      <c r="H23" s="3" t="inlineStr"/>
-      <c r="I23" s="3" t="inlineStr"/>
-      <c r="J23" s="3" t="inlineStr"/>
-      <c r="K23" s="3" t="inlineStr"/>
-      <c r="L23" s="3" t="inlineStr">
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
         <is>
           <t>Het antwoord staat letterlijk in de vraag ("vier cijfers plus twee letters").</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr"/>
-      <c r="N23" s="4" t="inlineStr">
+      <c r="M23" t="inlineStr"/>
+      <c r="N23" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O23" s="3" t="inlineStr"/>
-      <c r="P23" s="4" t="inlineStr"/>
-      <c r="Q23" s="3" t="inlineStr"/>
-      <c r="R23" s="3" t="inlineStr"/>
-      <c r="S23" s="3" t="inlineStr">
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr"/>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+      <c r="S23" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="n">
+      <c r="A24" t="n">
         <v>1155</v>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>Muziek</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E24" s="4" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Hoeveel bruggen telt het klassieke orkestnummer Bruggetje van Sainte Anneï in de titel niet?</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr"/>
-      <c r="G24" s="3" t="n">
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="n">
         <v>0</v>
       </c>
-      <c r="H24" s="3" t="inlineStr"/>
-      <c r="I24" s="3" t="inlineStr"/>
-      <c r="J24" s="3" t="inlineStr"/>
-      <c r="K24" s="3" t="inlineStr"/>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
         <is>
           <t>"Bruggetje van Sainte Anneï" bestaat niet; de vraag ontkent zichzelf.</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr"/>
-      <c r="N24" s="4" t="inlineStr">
+      <c r="M24" t="inlineStr"/>
+      <c r="N24" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O24" s="3" t="inlineStr"/>
-      <c r="P24" s="4" t="inlineStr"/>
-      <c r="Q24" s="3" t="inlineStr"/>
-      <c r="R24" s="3" t="inlineStr"/>
-      <c r="S24" s="3" t="inlineStr">
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr"/>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+      <c r="S24" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="n">
+      <c r="A25" t="n">
         <v>1156</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="D25" s="3" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E25" s="4" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Hoeveel dagen duurt de Alvleeskliervlaamse Wielerweek Vredeskoers niet?</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>How many days does the All-Flemish Wheeler Week Peace course not last?</t>
         </is>
       </c>
-      <c r="G25" s="3" t="n">
+      <c r="G25" t="n">
         <v>0</v>
       </c>
-      <c r="H25" s="3" t="inlineStr"/>
-      <c r="I25" s="3" t="inlineStr"/>
-      <c r="J25" s="3" t="inlineStr"/>
-      <c r="K25" s="3" t="inlineStr"/>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
         <is>
           <t>"Alvleeskliervlaamse Wielerweek" is verzonnen (alvleesklier = orgaan).</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr"/>
-      <c r="N25" s="4" t="inlineStr">
+      <c r="M25" t="inlineStr"/>
+      <c r="N25" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O25" s="3" t="inlineStr"/>
-      <c r="P25" s="4" t="inlineStr"/>
-      <c r="Q25" s="3" t="inlineStr"/>
-      <c r="R25" s="3" t="inlineStr"/>
-      <c r="S25" s="3" t="inlineStr">
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr"/>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="n">
+      <c r="A26" t="n">
         <v>1157</v>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
         <is>
           <t>Kunst en cultuur</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Hoeveel dagen duurt de Nederlands Dans Theater-productie Stop-Motion doorgaans per seizoensblok?</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>How many days does the Dutch Dance Theater production Stop-Motion usually last per seasonal block?</t>
         </is>
       </c>
-      <c r="G26" s="3" t="n">
+      <c r="G26" t="n">
         <v>3</v>
       </c>
-      <c r="H26" s="3" t="inlineStr"/>
-      <c r="I26" s="3" t="inlineStr"/>
-      <c r="J26" s="3" t="inlineStr"/>
-      <c r="K26" s="3" t="inlineStr"/>
-      <c r="L26" s="3" t="inlineStr">
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
         <is>
           <t>Verzonnen meeteenheid: "per seizoensblok".</t>
         </is>
       </c>
-      <c r="M26" s="3" t="inlineStr"/>
-      <c r="N26" s="4" t="inlineStr">
+      <c r="M26" t="inlineStr"/>
+      <c r="N26" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O26" s="3" t="inlineStr"/>
-      <c r="P26" s="4" t="inlineStr"/>
-      <c r="Q26" s="3" t="inlineStr"/>
-      <c r="R26" s="3" t="inlineStr"/>
-      <c r="S26" s="3" t="inlineStr">
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr"/>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+      <c r="S26" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="n">
+      <c r="A27" t="n">
         <v>1163</v>
       </c>
-      <c r="B27" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>Economie &amp; geld</t>
         </is>
       </c>
-      <c r="D27" s="3" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E27" s="4" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Hoeveel eenheden telt de Nederlandse duizendguldenbiljet-collectie uit 1970?</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>How many units does the 1970 Dutch thousand guilder banknote collection have?</t>
         </is>
       </c>
-      <c r="G27" s="3" t="n">
+      <c r="G27" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="3" t="inlineStr"/>
-      <c r="I27" s="3" t="inlineStr"/>
-      <c r="J27" s="3" t="inlineStr"/>
-      <c r="K27" s="3" t="inlineStr"/>
-      <c r="L27" s="3" t="inlineStr">
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
         <is>
           <t>Verzonnen: er bestaat geen "duizendguldenbiljet-collectie uit 1970".</t>
         </is>
       </c>
-      <c r="M27" s="3" t="inlineStr"/>
-      <c r="N27" s="4" t="inlineStr">
+      <c r="M27" t="inlineStr"/>
+      <c r="N27" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O27" s="3" t="inlineStr"/>
-      <c r="P27" s="4" t="inlineStr">
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
         <is>
           <t>"De duizendguldenbiljet-collectie uit 1970" bestaat niet als begrip, en het antwoord een maakt elke deelsom stuk.</t>
         </is>
       </c>
-      <c r="Q27" s="3" t="inlineStr"/>
-      <c r="R27" s="3" t="inlineStr"/>
-      <c r="S27" s="3" t="inlineStr">
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+      <c r="S27" t="inlineStr">
         <is>
           <t>vraag deugt niet (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="n">
+      <c r="A28" t="n">
         <v>1170</v>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>Hoeveel gram boter gaat in de klassieke Nederlandse boterkoek per 10 porties?</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>How many grams of butter goes into the classic Dutch buttercake per 10 portions?</t>
         </is>
       </c>
-      <c r="G28" s="3" t="n">
+      <c r="G28" t="n">
         <v>250</v>
       </c>
-      <c r="H28" s="3" t="inlineStr"/>
-      <c r="I28" s="3" t="inlineStr"/>
-      <c r="J28" s="3" t="inlineStr"/>
-      <c r="K28" s="3" t="inlineStr"/>
-      <c r="L28" s="3" t="inlineStr"/>
-      <c r="M28" s="3" t="inlineStr"/>
-      <c r="N28" s="4" t="inlineStr">
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O28" s="3" t="inlineStr"/>
-      <c r="P28" s="4" t="inlineStr"/>
-      <c r="Q28" s="3" t="inlineStr"/>
-      <c r="R28" s="3" t="inlineStr"/>
-      <c r="S28" s="3" t="inlineStr">
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr"/>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+      <c r="S28" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="n">
+      <c r="A29" t="n">
         <v>1171</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="D29" s="3" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E29" s="4" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>Hoeveel gram suiker bevat een standaard reep chocolade van Droste van 100 gram ongeveer?</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr"/>
-      <c r="G29" s="3" t="n">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="n">
         <v>55</v>
       </c>
-      <c r="H29" s="3" t="inlineStr"/>
-      <c r="I29" s="3" t="inlineStr"/>
-      <c r="J29" s="3" t="inlineStr"/>
-      <c r="K29" s="3" t="inlineStr"/>
-      <c r="L29" s="3" t="inlineStr"/>
-      <c r="M29" s="3" t="inlineStr"/>
-      <c r="N29" s="4" t="inlineStr">
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O29" s="3" t="inlineStr"/>
-      <c r="P29" s="4" t="inlineStr"/>
-      <c r="Q29" s="3" t="inlineStr"/>
-      <c r="R29" s="3" t="inlineStr"/>
-      <c r="S29" s="3" t="inlineStr">
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr"/>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+      <c r="S29" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="n">
+      <c r="A30" t="n">
         <v>1172</v>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
         <is>
           <t>Eten &amp; drinken</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D30" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E30" s="4" t="inlineStr">
+      <c r="E30" t="inlineStr">
         <is>
           <t>Hoeveel gram weegt een stroopwafel van het merk Daelmans standaard?</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="F30" t="inlineStr">
         <is>
           <t>How many grams does a syrup waffle of the Daelmans standard weigh?</t>
         </is>
       </c>
-      <c r="G30" s="3" t="n">
+      <c r="G30" t="n">
         <v>32</v>
       </c>
-      <c r="H30" s="3" t="inlineStr"/>
-      <c r="I30" s="3" t="inlineStr"/>
-      <c r="J30" s="3" t="inlineStr"/>
-      <c r="K30" s="3" t="inlineStr"/>
-      <c r="L30" s="3" t="inlineStr"/>
-      <c r="M30" s="3" t="inlineStr"/>
-      <c r="N30" s="4" t="inlineStr">
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O30" s="3" t="inlineStr"/>
-      <c r="P30" s="4" t="inlineStr"/>
-      <c r="Q30" s="3" t="inlineStr"/>
-      <c r="R30" s="3" t="inlineStr"/>
-      <c r="S30" s="3" t="inlineStr">
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr"/>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+      <c r="S30" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="n">
+      <c r="A31" t="n">
         <v>1175</v>
       </c>
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="inlineStr">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>Spellen en speelgoed</t>
         </is>
       </c>
-      <c r="D31" s="3" t="inlineStr">
+      <c r="D31" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E31" s="4" t="inlineStr">
+      <c r="E31" t="inlineStr">
         <is>
           <t>Hoeveel kapstokkaarten telt een standaard Nederlandse Mens-erger-je-niet?</t>
         </is>
       </c>
-      <c r="F31" s="3" t="inlineStr">
+      <c r="F31" t="inlineStr">
         <is>
           <t>How many card cards does a standard Dutch Mens-erger-je-not have?</t>
         </is>
       </c>
-      <c r="G31" s="3" t="n">
+      <c r="G31" t="n">
         <v>4</v>
       </c>
-      <c r="H31" s="3" t="inlineStr"/>
-      <c r="I31" s="3" t="inlineStr"/>
-      <c r="J31" s="3" t="inlineStr"/>
-      <c r="K31" s="3" t="inlineStr"/>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
         <is>
           <t>"Kapstokkaarten" bestaan niet in Mens-erger-je-niet.</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr"/>
-      <c r="N31" s="4" t="inlineStr">
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O31" s="3" t="inlineStr"/>
-      <c r="P31" s="4" t="inlineStr"/>
-      <c r="Q31" s="3" t="inlineStr"/>
-      <c r="R31" s="3" t="inlineStr"/>
-      <c r="S31" s="3" t="inlineStr">
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr"/>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+      <c r="S31" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="3" t="n">
+      <c r="A32" t="n">
         <v>1177</v>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>Dagelijks leven</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E32" s="4" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Hoeveel keer per jaar publiceert het CBS de driejaarlijkse woondenquête?</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>How many times a year does the CBS publish the three-yearly living survey?</t>
         </is>
       </c>
-      <c r="G32" s="3" t="n">
+      <c r="G32" t="n">
         <v>1</v>
       </c>
-      <c r="H32" s="3" t="inlineStr"/>
-      <c r="I32" s="3" t="inlineStr"/>
-      <c r="J32" s="3" t="inlineStr"/>
-      <c r="K32" s="3" t="inlineStr"/>
-      <c r="L32" s="3" t="inlineStr">
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
         <is>
           <t>Spreekt zichzelf tegen: "per jaar" versus "driejaarlijkse".</t>
         </is>
       </c>
-      <c r="M32" s="3" t="inlineStr"/>
-      <c r="N32" s="4" t="inlineStr">
+      <c r="M32" t="inlineStr"/>
+      <c r="N32" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O32" s="3" t="inlineStr"/>
-      <c r="P32" s="4" t="inlineStr"/>
-      <c r="Q32" s="3" t="inlineStr"/>
-      <c r="R32" s="3" t="inlineStr"/>
-      <c r="S32" s="3" t="inlineStr">
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr"/>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="n">
+      <c r="A33" t="n">
         <v>1198</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
         <is>
           <t>Politiek en recht</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>Hoeveel koppen bevat de Nederlandse driehoek bestuursniveaus (rijk, provincie, gemeente)?</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F33" t="inlineStr">
         <is>
           <t>How many headlines does the Dutch triangle contain levels of government (rich, province, municipality)?</t>
         </is>
       </c>
-      <c r="G33" s="3" t="n">
+      <c r="G33" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="3" t="inlineStr"/>
-      <c r="I33" s="3" t="inlineStr"/>
-      <c r="J33" s="3" t="inlineStr"/>
-      <c r="K33" s="3" t="inlineStr"/>
-      <c r="L33" s="3" t="inlineStr">
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr">
         <is>
           <t>"Koppen" is hier onzin; het antwoord staat in de vraag.</t>
         </is>
       </c>
-      <c r="M33" s="3" t="inlineStr"/>
-      <c r="N33" s="4" t="inlineStr">
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O33" s="3" t="inlineStr"/>
-      <c r="P33" s="4" t="inlineStr"/>
-      <c r="Q33" s="3" t="inlineStr"/>
-      <c r="R33" s="3" t="inlineStr"/>
-      <c r="S33" s="3" t="inlineStr">
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr"/>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="3" t="n">
+      <c r="A34" t="n">
         <v>1203</v>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>Geschiedenis</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Nederlands</t>
         </is>
       </c>
-      <c r="E34" s="4" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Hoeveel landen kocht de VOC formeel aan als koloniale gebieden?</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr"/>
-      <c r="G34" s="3" t="n">
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="n">
         <v>0</v>
       </c>
-      <c r="H34" s="3" t="inlineStr"/>
-      <c r="I34" s="3" t="inlineStr"/>
-      <c r="J34" s="3" t="inlineStr"/>
-      <c r="K34" s="3" t="inlineStr"/>
-      <c r="L34" s="3" t="inlineStr">
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
         <is>
           <t>De VOC kocht geen landen; feitelijk onjuiste premisse.</t>
         </is>
       </c>
-      <c r="M34" s="3" t="inlineStr"/>
-      <c r="N34" s="4" t="inlineStr">
+      <c r="M34" t="inlineStr"/>
+      <c r="N34" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O34" s="3" t="inlineStr"/>
-      <c r="P34" s="4" t="inlineStr"/>
-      <c r="Q34" s="3" t="inlineStr"/>
-      <c r="R34" s="3" t="inlineStr"/>
-      <c r="S34" s="3" t="inlineStr">
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr"/>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="n">
+      <c r="A35" t="n">
         <v>1258</v>
       </c>
-      <c r="B35" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>Politiek en recht</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>Politiek en recht</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>Hoeveel emiraten heeft Saoedi-Arabië als koninkrijk in bestuurlijke regio (provincies)?</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F35" t="inlineStr">
         <is>
           <t>How many emirates has Saudi Arabia as a kingdom in administrative region (provincies)?</t>
         </is>
       </c>
-      <c r="G35" s="3" t="n">
+      <c r="G35" t="n">
         <v>13</v>
       </c>
-      <c r="H35" s="3" t="inlineStr"/>
-      <c r="I35" s="3" t="inlineStr"/>
-      <c r="J35" s="3" t="inlineStr"/>
-      <c r="K35" s="3" t="inlineStr"/>
-      <c r="L35" s="3" t="inlineStr">
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr">
         <is>
           <t>Feitelijk onjuist: Saoedi-Arabië heeft geen emiraten.</t>
         </is>
       </c>
-      <c r="M35" s="3" t="inlineStr"/>
-      <c r="N35" s="4" t="inlineStr">
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O35" s="3" t="inlineStr"/>
-      <c r="P35" s="4" t="inlineStr"/>
-      <c r="Q35" s="3" t="inlineStr"/>
-      <c r="R35" s="3" t="inlineStr"/>
-      <c r="S35" s="3" t="inlineStr">
+      <c r="O35" t="inlineStr"/>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr"/>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="3" t="n">
+      <c r="A36" t="n">
         <v>1287</v>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
         <is>
           <t>Politiek en recht</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D36" t="inlineStr">
         <is>
           <t>Politiek en recht</t>
         </is>
       </c>
-      <c r="E36" s="4" t="inlineStr">
+      <c r="E36" t="inlineStr">
         <is>
           <t>Hoeveel rechterzittingen telt het Amerikaanse Hooggerechtshof?</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
+      <c r="F36" t="inlineStr">
         <is>
           <t>How many court hearings does the U.S. Supreme Court have?</t>
         </is>
       </c>
-      <c r="G36" s="3" t="n">
+      <c r="G36" t="n">
         <v>9</v>
       </c>
-      <c r="H36" s="3" t="inlineStr"/>
-      <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="3" t="inlineStr"/>
-      <c r="K36" s="3" t="inlineStr"/>
-      <c r="L36" s="3" t="inlineStr">
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr">
         <is>
           <t>Vraagt naar "rechterzittingen"; bedoeld is het aantal rechters.</t>
         </is>
       </c>
-      <c r="M36" s="3" t="inlineStr"/>
-      <c r="N36" s="4" t="inlineStr">
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O36" s="3" t="inlineStr"/>
-      <c r="P36" s="4" t="inlineStr"/>
-      <c r="Q36" s="3" t="inlineStr"/>
-      <c r="R36" s="3" t="inlineStr"/>
-      <c r="S36" s="3" t="inlineStr">
+      <c r="O36" t="inlineStr"/>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr"/>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="3" t="n">
+      <c r="A37" t="n">
         <v>1374</v>
       </c>
-      <c r="B37" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="D37" s="3" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="E37" s="4" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>Hoeveel kuiven heeft een honkbalveld (bases plus home plate)?</t>
         </is>
       </c>
-      <c r="F37" s="3" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>How many coves has a baseball field (bases plus home plates)?</t>
         </is>
       </c>
-      <c r="G37" s="3" t="n">
+      <c r="G37" t="n">
         <v>4</v>
       </c>
-      <c r="H37" s="3" t="inlineStr"/>
-      <c r="I37" s="3" t="inlineStr"/>
-      <c r="J37" s="3" t="inlineStr"/>
-      <c r="K37" s="3" t="inlineStr"/>
-      <c r="L37" s="3" t="inlineStr">
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr"/>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr">
         <is>
           <t>"Kuiven" bestaat niet in deze betekenis; bedoeld zijn honkholtes of bases.</t>
         </is>
       </c>
-      <c r="M37" s="3" t="inlineStr"/>
-      <c r="N37" s="4" t="inlineStr">
+      <c r="M37" t="inlineStr"/>
+      <c r="N37" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O37" s="3" t="inlineStr"/>
-      <c r="P37" s="4" t="inlineStr"/>
-      <c r="Q37" s="3" t="inlineStr"/>
-      <c r="R37" s="3" t="inlineStr"/>
-      <c r="S37" s="3" t="inlineStr">
+      <c r="O37" t="inlineStr"/>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr"/>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="3" t="n">
+      <c r="A38" t="n">
         <v>1394</v>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Hoeveel proloog kilometers telt een Tour de France etappe bijna nooit?</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr"/>
-      <c r="G38" s="3" t="n">
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="n">
         <v>0</v>
       </c>
-      <c r="H38" s="3" t="inlineStr"/>
-      <c r="I38" s="3" t="inlineStr"/>
-      <c r="J38" s="3" t="inlineStr"/>
-      <c r="K38" s="3" t="inlineStr"/>
-      <c r="L38" s="3" t="inlineStr">
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr">
         <is>
           <t>Dubbele ontkenning ("telt een etappe bijna nooit") maakt het onbeantwoordbaar.</t>
         </is>
       </c>
-      <c r="M38" s="3" t="inlineStr"/>
-      <c r="N38" s="4" t="inlineStr">
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O38" s="3" t="inlineStr"/>
-      <c r="P38" s="4" t="inlineStr"/>
-      <c r="Q38" s="3" t="inlineStr"/>
-      <c r="R38" s="3" t="inlineStr"/>
-      <c r="S38" s="3" t="inlineStr">
+      <c r="O38" t="inlineStr"/>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr"/>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr">
         <is>
           <t>geen bron mogelijk (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="n">
+      <c r="A39" t="n">
         <v>1400</v>
       </c>
-      <c r="B39" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="D39" s="3" t="inlineStr">
+      <c r="D39" t="inlineStr">
         <is>
           <t>Sport</t>
         </is>
       </c>
-      <c r="E39" s="4" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>Hoeveel rings heeft het NBA-logo in het midden?</t>
         </is>
       </c>
-      <c r="F39" s="3" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>How many rings does the NBA logo have in the middle?</t>
         </is>
       </c>
-      <c r="G39" s="3" t="n">
+      <c r="G39" t="n">
         <v>1</v>
       </c>
-      <c r="H39" s="3" t="inlineStr"/>
-      <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="3" t="inlineStr"/>
-      <c r="K39" s="3" t="inlineStr"/>
-      <c r="L39" s="3" t="inlineStr">
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr"/>
+      <c r="K39" t="inlineStr"/>
+      <c r="L39" t="inlineStr">
         <is>
           <t>"Rings" is Engels blijven staan; het NBA-logo heeft geen ringen.</t>
         </is>
       </c>
-      <c r="M39" s="3" t="inlineStr"/>
-      <c r="N39" s="4" t="inlineStr">
+      <c r="M39" t="inlineStr"/>
+      <c r="N39" t="inlineStr">
         <is>
           <t>geen bron</t>
         </is>
       </c>
-      <c r="O39" s="3" t="inlineStr"/>
-      <c r="P39" s="4" t="inlineStr">
+      <c r="O39" t="inlineStr"/>
+      <c r="P39" t="inlineStr">
         <is>
           <t>Het NBA-logo is een silhouet van een basketballer en heeft geen ringen. De vraag klopt niet, en het antwoord een maakt elke deelsom stuk.</t>
         </is>
       </c>
-      <c r="Q39" s="3" t="inlineStr"/>
-      <c r="R39" s="3" t="inlineStr"/>
-      <c r="S39" s="3" t="inlineStr">
+      <c r="Q39" t="inlineStr"/>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr">
         <is>
           <t>vraag deugt niet (onbruikbaar)</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="3" t="n">
+      <c r="A40" t="n">
         <v>1457</v>
       </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
         <is>
           <t>Technologie</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D40" t="inlineStr">
         <is>
           <t>Technologie</t>
         </is>
       </c>
-      <c r="E40" s="4" t="inlineStr">
+      <c r="E40" t="inlineStr">
         <is>
           <t>Hoeveel megabytes zitten er in precies één gigabyte?</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr"/>
-      <c r="G40" s="3" t="n">
+      <c r="F40" t="inlineStr"/>
+      <c r="G40" t="n">
         <v>1024</v>
       </c>
-      <c r="H40" s="3" t="inlineStr">
+      <c r="H40" t="inlineStr">
         <is>
           <t>https://physics.nist.gov/cuu/Units/binary.html</t>
         </is>
       </c>
-      <c r="I40" s="3" t="inlineStr"/>
-      <c r="J40" s="3" t="inlineStr"/>
-      <c r="K40" s="3" t="inlineStr"/>
-      <c r="L40" s="3" t="inlineStr"/>
-      <c r="M40" s="3" t="inlineStr"/>
-      <c r="N40" s="4" t="inlineStr">
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr"/>
+      <c r="K40" t="inlineStr"/>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr"/>
+      <c r="N40" t="inlineStr">
         <is>
           <t>Vraagt hoeveel megabyte in "precies een gigabyte" gaan; dat zijn er 1000, niet 1024. Vraag 1458 stelt dezelfde vraag mét de binaire voorwaarde en is daarmee correct. Deze vraag is een dubbele met een fout antwoord.</t>
         </is>
       </c>
-      <c r="O40" s="3" t="inlineStr">
+      <c r="O40" t="inlineStr">
         <is>
           <t>https://physics.nist.gov/cuu/Units/binary.html</t>
         </is>
       </c>
-      <c r="P40" s="4" t="inlineStr">
+      <c r="P40" t="inlineStr">
         <is>
           <t>De vraag zegt "precies een gigabyte", en dan is het antwoord 1000 megabyte. De 1024 hoort bij de gibibyte. Vraag 1458 stelt dezelfde vraag wel goed.</t>
         </is>
       </c>
-      <c r="Q40" s="3" t="inlineStr"/>
-      <c r="R40" s="3" t="inlineStr">
+      <c r="Q40" t="inlineStr"/>
+      <c r="R40" t="inlineStr">
         <is>
           <t>onbruikbaar</t>
         </is>
       </c>
-      <c r="S40" s="3" t="inlineStr">
+      <c r="S40" t="inlineStr">
         <is>
           <t>vraag vervallen</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="3" t="n">
+      <c r="A41" t="n">
         <v>1472</v>
       </c>
-      <c r="B41" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
         <is>
           <t>Technologie</t>
         </is>
       </c>
-      <c r="D41" s="3" t="inlineStr">
+      <c r="D41" t="inlineStr">
         <is>
           <t>Technologie</t>
         </is>
       </c>
-      <c r="E41" s="4" t="inlineStr">
+      <c r="E41" t="inlineStr">
         <is>
           <t>In welk jaar werd de Toyota motorfiets eerste gebouwd - nee Toyota is auto (1885 Daimler - dit zit niet in Azië)?</t>
         </is>
       </c>
-      <c r="F41" s="3" t="inlineStr"/>
-      <c r="G41" s="3" t="n">
+      <c r="F41" t="inlineStr"/>
+      <c r="G41" t="n">
         <v>0</v>
       </c>
-      <c r="H41" s="3" t="inlineStr"/>
-      <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="3" t="inlineStr"/>
-      <c r="K41" s="3" t="inlineStr"/>
-      <c r="L41" s="3" t="inlineStr">
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr"/>
+      <c r="K41" t="inlineStr"/>
+      <c r="L41" t="inlineStr">
         <is>
           <t>Bevat de redactienotitie "nee Toyota is auto (1885 Daimler - dit zit niet in Azië)".</t>
         </is>
       </c>
-      <c r="M41" s="3" t="inlineStr"/>
-      <c r="N41" s="4" t="inlineStr">
+      <c r="M41" t="inlineStr"/>
+      <c r="N41" t="inlineStr">
         <is>
           <t>geen bron · geen EN-vertaling</t>
         </is>
       </c>
-      <c r="O41" s="3" t="inlineStr"/>
-      <c r="P41" s="4" t="inlineStr"/>
-      <c r="Q41" s="3" t="inlineStr"/>
-      <c r="R41" s="3" t="inlineStr"/>
-      <c r="S41" s="3" t="inlineStr">
-        <is>
-          <t>geen bron mogelijk (onbruikbaar)</t>
-        </is>
-      </c>
+      <c r="O41" t="inlineStr"/>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr"/>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>geen bron mogelijk (onbruikbaar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>1063</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Kunst en cultuur</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Kunst en cultuur</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Hoeveel natuursonden (beelden) staan er op Paaseiland - sorry dat zit niet in Europa!</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>How many scenes of nature are there on Easter Island - sorry that's not in Europe!</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr"/>
+      <c r="K42" t="inlineStr"/>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Bevat de redactienotitie "sorry dat zit niet in Europa!"; "natuursonden" is bovendien geen woord.</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr"/>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>geen bron</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>https://nl.wikipedia.org/wiki/Paaseiland</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>Bahn (2002), The enigma's of Easter Island, Oxford University Press, ISBN 0-19-280340-9
+Externe link
+(en)  Korte documentaire van David Attenborough over Paaseiland
+Referenties</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr"/>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>1164</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Geografie</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Nederlands</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Hoeveel eilanden telt de Nederlandse Antillen in de huidige status van landen?</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr"/>
+      <c r="G43" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr"/>
+      <c r="K43" t="inlineStr"/>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr"/>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>geen bron · geen EN-vertaling</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>https://nl.wikipedia.org/wiki/Nederlandse_Antillen</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>De leeftijdsopbouw was:
+0-14 jaar 23,9%
+15-65 jaar 67,3%
+66 jaar en ouder 8,7%
+De levensverwachting was:
+Totale bevolking 76,03 jaar
+Mannen 73,76 jaar
+Vrouwen 78,41 jaar
+De Nederlandse Antillen had een bevolkingsgroei van 0,79%.</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr"/>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>1201</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Sport</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Nederlands</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Hoeveel landen deden er mee aan het Nederlands kampioenschap wielrennen voor clubs?</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>How many countries participated in the Dutch cycling championship for clubs?</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr"/>
+      <c r="K44" t="inlineStr"/>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Een nationaal kampioenschap heeft per definitie één land.</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr"/>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>geen bron</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>https://nl.wikipedia.org/wiki/Nederlands</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>Het Nederlands alleen wordt door meer mensen gesproken dan de Noord-Germaanse (Scandinavische) talen bij elkaar: Zweeds (10 miljoen), Noors (5 miljoen), Deens (5 miljoen) en IJslands (0,3 miljoen).</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr"/>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>1204</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Politiek en recht</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Nederlands</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Hoeveel landen stemden vóór het Nederlands als EU-taal?</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr"/>
+      <c r="K45" t="inlineStr"/>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Verzonnen stemming; zo werkt de EU-talenregeling niet.</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr"/>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>geen bron · geen EN-vertaling</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>https://nl.wikipedia.org/wiki/Nederlands</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>Het Nederlands alleen wordt door meer mensen gesproken dan de Noord-Germaanse (Scandinavische) talen bij elkaar: Zweeds (10 miljoen), Noors (5 miljoen), Deens (5 miljoen) en IJslands (0,3 miljoen).</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr"/>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>1324</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Scheikunde</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Scheikunde</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Hoeveel graden Celsius is het vriespunt van water bij normale luchtdruk?</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>How many degrees Celsius is the freezing point of water at normal air pressure?</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>https://webbook.nist.gov/cgi/cbook.cgi?ID=C7732185</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr"/>
+      <c r="K46" t="inlineStr"/>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr"/>
+      <c r="N46" t="inlineStr"/>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>https://nl.wikipedia.org/wiki/Celsius</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>De celsiusschaal is gedefinieerd met de volgende twee ijkpunten:
+0 °C (0 graden Celsius) is de temperatuur waarbij water bevriest bij een luchtdruk van 1 atmosfeer.</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr"/>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>hoog</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>